<commit_message>
feat: massive performance optimization for production scale
</commit_message>
<xml_diff>
--- a/backend/_data_list/users.xlsx
+++ b/backend/_data_list/users.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04\home\neelima\projects\Orange-Flow-Next-Js\backend\_data_list\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Telegram_Project\Orange-Flow-Next-Js\backend\_data_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F248ED3-8E66-461A-A578-18B672D29EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C244B4-19DE-46B7-9C4E-96B4EBE94B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BB0F9CCB-0FBE-4AFF-BD3B-D4E64BAEDA77}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BB0F9CCB-0FBE-4AFF-BD3B-D4E64BAEDA77}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -675,20 +675,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B226F8CE-143F-43E3-8E7D-9AF252188EC1}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultColWidth="13.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="13.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -717,7 +717,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>8704561358</v>
       </c>
@@ -746,7 +746,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>8759226993</v>
       </c>
@@ -775,7 +775,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>8474847602</v>
       </c>
@@ -804,7 +804,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>8217920077</v>
       </c>
@@ -833,7 +833,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>8251541258</v>
       </c>
@@ -862,7 +862,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6857806283</v>
       </c>
@@ -891,7 +891,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>8434757540</v>
       </c>
@@ -920,7 +920,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7891698602</v>
       </c>
@@ -949,7 +949,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8681308050</v>
       </c>
@@ -978,7 +978,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>6287137090</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>6594315783</v>
       </c>
@@ -1036,7 +1036,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>7524803812</v>
       </c>
@@ -1065,7 +1065,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>7479560514</v>
       </c>
@@ -1094,7 +1094,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>7224463249</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>6519999519</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>7586404983</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>7713329612</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>8273936271</v>
       </c>
@@ -1239,7 +1239,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>8980795758</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>6534313772</v>
       </c>
@@ -1297,16 +1297,16 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E25" s="1"/>
     </row>
   </sheetData>

</xml_diff>